<commit_message>
numerous updates to fertility analysis and ran zr mixing at 10,000
</commit_message>
<xml_diff>
--- a/Mataquito/MataquitoSampleData.xlsx
+++ b/Mataquito/MataquitoSampleData.xlsx
@@ -1,19 +1,20 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11122"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10215"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/Glong1/Desktop/Andes/AndesTG/Mataquito/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B26892DE-5401-0A4E-BA0F-5001B932562B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9EF0CC73-A75E-5748-AB57-F270E85CD1A1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="620" windowWidth="38400" windowHeight="21860" xr2:uid="{822C4A32-E1B2-FB43-A333-01FAD55EB50E}"/>
+    <workbookView xWindow="0" yWindow="620" windowWidth="38400" windowHeight="21860" activeTab="1" xr2:uid="{822C4A32-E1B2-FB43-A333-01FAD55EB50E}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="Sheet2" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="181029"/>
   <extLst>
@@ -36,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="44" uniqueCount="33">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="62" uniqueCount="33">
   <si>
     <t>Latitude</t>
   </si>
@@ -1213,55 +1214,6 @@
       </c>
     </row>
     <row r="14" spans="1:27" x14ac:dyDescent="0.2">
-      <c r="A14" s="1" t="s">
-        <v>30</v>
-      </c>
-      <c r="B14" s="1" t="s">
-        <v>31</v>
-      </c>
-      <c r="C14" s="1">
-        <v>-35.056683</v>
-      </c>
-      <c r="D14" s="1">
-        <v>-72.163951999999995</v>
-      </c>
-      <c r="F14" s="1">
-        <v>9</v>
-      </c>
-      <c r="G14" s="2">
-        <v>1451.47</v>
-      </c>
-      <c r="H14" s="1"/>
-      <c r="I14" s="1">
-        <v>1</v>
-      </c>
-      <c r="J14" s="1">
-        <v>17.15361</v>
-      </c>
-      <c r="K14" s="1">
-        <v>8.6699999999999999E-2</v>
-      </c>
-      <c r="L14" s="3">
-        <v>1.53E-13</v>
-      </c>
-      <c r="M14" s="3">
-        <v>2.8599999999999999E-15</v>
-      </c>
-      <c r="N14" s="3">
-        <v>51000</v>
-      </c>
-      <c r="O14" s="3">
-        <v>967</v>
-      </c>
-      <c r="P14" s="1">
-        <v>91.6</v>
-      </c>
-      <c r="Q14" s="1">
-        <v>8</v>
-      </c>
-      <c r="R14" s="1">
-        <v>10.8</v>
-      </c>
       <c r="S14" s="1"/>
       <c r="T14" s="1"/>
       <c r="U14" s="1"/>
@@ -1273,55 +1225,6 @@
       <c r="AA14" s="1"/>
     </row>
     <row r="15" spans="1:27" x14ac:dyDescent="0.2">
-      <c r="A15" s="1" t="s">
-        <v>32</v>
-      </c>
-      <c r="B15" s="1" t="s">
-        <v>31</v>
-      </c>
-      <c r="C15" s="1">
-        <v>-35.055520999999999</v>
-      </c>
-      <c r="D15" s="1">
-        <v>-72.163645000000002</v>
-      </c>
-      <c r="F15" s="1">
-        <v>9</v>
-      </c>
-      <c r="G15" s="2">
-        <v>1451.47</v>
-      </c>
-      <c r="H15" s="1"/>
-      <c r="I15" s="1">
-        <v>1</v>
-      </c>
-      <c r="J15" s="1">
-        <v>11.14916</v>
-      </c>
-      <c r="K15" s="1">
-        <v>8.5999999999999993E-2</v>
-      </c>
-      <c r="L15" s="3">
-        <v>2.3400000000000001E-13</v>
-      </c>
-      <c r="M15" s="3">
-        <v>4.3500000000000001E-15</v>
-      </c>
-      <c r="N15" s="3">
-        <v>120000</v>
-      </c>
-      <c r="O15" s="3">
-        <v>2250</v>
-      </c>
-      <c r="P15" s="1">
-        <v>49.4</v>
-      </c>
-      <c r="Q15" s="1">
-        <v>2.42</v>
-      </c>
-      <c r="R15" s="1">
-        <v>4.62</v>
-      </c>
       <c r="S15" s="1"/>
       <c r="T15" s="1"/>
       <c r="U15" s="1"/>
@@ -1335,4 +1238,174 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{94D41E08-87A4-684F-84A3-DF79FCDB8B3A}">
+  <dimension ref="A1:R3"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <sheetData>
+    <row r="1" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="A1" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="H1" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="I1" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="J1" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="K1" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="L1" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="M1" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="N1" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="O1" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="P1" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="Q1" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="R1" s="1" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="2" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="A2" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="C2" s="1">
+        <v>-35.056683</v>
+      </c>
+      <c r="D2" s="1">
+        <v>-72.163951999999995</v>
+      </c>
+      <c r="E2" s="1"/>
+      <c r="F2" s="1">
+        <v>9</v>
+      </c>
+      <c r="G2" s="2">
+        <v>1451.47</v>
+      </c>
+      <c r="H2" s="1"/>
+      <c r="I2" s="1">
+        <v>1</v>
+      </c>
+      <c r="J2" s="1">
+        <v>17.15361</v>
+      </c>
+      <c r="K2" s="1">
+        <v>8.6699999999999999E-2</v>
+      </c>
+      <c r="L2" s="3">
+        <v>1.53E-13</v>
+      </c>
+      <c r="M2" s="3">
+        <v>2.8599999999999999E-15</v>
+      </c>
+      <c r="N2" s="3">
+        <v>51000</v>
+      </c>
+      <c r="O2" s="3">
+        <v>967</v>
+      </c>
+      <c r="P2" s="1">
+        <v>91.6</v>
+      </c>
+      <c r="Q2" s="1">
+        <v>8</v>
+      </c>
+      <c r="R2" s="1">
+        <v>10.8</v>
+      </c>
+    </row>
+    <row r="3" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="A3" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="B3" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="C3" s="1">
+        <v>-35.055520999999999</v>
+      </c>
+      <c r="D3" s="1">
+        <v>-72.163645000000002</v>
+      </c>
+      <c r="E3" s="1"/>
+      <c r="F3" s="1">
+        <v>9</v>
+      </c>
+      <c r="G3" s="2">
+        <v>1451.47</v>
+      </c>
+      <c r="H3" s="1"/>
+      <c r="I3" s="1">
+        <v>1</v>
+      </c>
+      <c r="J3" s="1">
+        <v>11.14916</v>
+      </c>
+      <c r="K3" s="1">
+        <v>8.5999999999999993E-2</v>
+      </c>
+      <c r="L3" s="3">
+        <v>2.3400000000000001E-13</v>
+      </c>
+      <c r="M3" s="3">
+        <v>4.3500000000000001E-15</v>
+      </c>
+      <c r="N3" s="3">
+        <v>120000</v>
+      </c>
+      <c r="O3" s="3">
+        <v>2250</v>
+      </c>
+      <c r="P3" s="1">
+        <v>49.4</v>
+      </c>
+      <c r="Q3" s="1">
+        <v>2.42</v>
+      </c>
+      <c r="R3" s="1">
+        <v>4.62</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>